<commit_message>
Readability and Ease-of-Use Changes
- Deleted data_analysis_workbook.ipynb as this was converted to separate py files.
- Deleted question_database_schema in main folder as all calls should be made from /data/question_database_schema.xlsx
- Deleted export_student_response_data.py, read_pdf_data as this was specific to converting our raw data and is not useful generally.
- Added results folder in main dir. Moved all calculated statistics there.
- Added misc folder to main dir and moved ICC_viz.ipynb as this was an image just generated for the paper and not applicable for the methodology.
- Updated README.md to explain how to use scripts.
</commit_message>
<xml_diff>
--- a/corr_matrix/residual_exam3C_1PL.xlsx
+++ b/corr_matrix/residual_exam3C_1PL.xlsx
@@ -1,37 +1,96 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="17">
+  <si>
+    <t>3C02</t>
+  </si>
+  <si>
+    <t>3C03</t>
+  </si>
+  <si>
+    <t>3C04</t>
+  </si>
+  <si>
+    <t>3C05</t>
+  </si>
+  <si>
+    <t>3C06</t>
+  </si>
+  <si>
+    <t>3C07</t>
+  </si>
+  <si>
+    <t>3C08</t>
+  </si>
+  <si>
+    <t>3C09</t>
+  </si>
+  <si>
+    <t>3C10</t>
+  </si>
+  <si>
+    <t>3C11</t>
+  </si>
+  <si>
+    <t>3C12</t>
+  </si>
+  <si>
+    <t>3C13</t>
+  </si>
+  <si>
+    <t>3C14</t>
+  </si>
+  <si>
+    <t>3C15</t>
+  </si>
+  <si>
+    <t>3C16</t>
+  </si>
+  <si>
+    <t>3C17</t>
+  </si>
+  <si>
+    <t>question_id</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,93 +105,35 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -420,982 +421,912 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>question_id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>3C02</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>3C03</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>3C04</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>3C05</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>3C06</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>3C07</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>3C08</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>3C09</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>3C10</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>3C11</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>3C12</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>3C13</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>3C14</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>3C15</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>3C16</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>3C17</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>3C02</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" t="n">
+    <row r="1" spans="1:17">
+      <c r="A1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
         <v>0.04750649153851164</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>-0.1121271029347614</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>0.01467795809162198</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>-0.0998038780137567</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2">
         <v>-0.2055615731357613</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2">
         <v>0.03873230532879787</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2">
         <v>0.002201016425689495</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2">
         <v>-0.1213430151999095</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2">
         <v>0.06225760883671789</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2">
         <v>-0.231502533472337</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M2">
         <v>0.0622219564254666</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2">
         <v>-0.07143255158646721</v>
       </c>
-      <c r="O2" t="n">
+      <c r="O2">
         <v>0.2287020214566456</v>
       </c>
-      <c r="P2" t="n">
+      <c r="P2">
         <v>-0.0286133563571018</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="Q2">
         <v>-0.1376742995782222</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>3C03</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+    <row r="3" spans="1:17">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
         <v>0.04750649153851164</v>
       </c>
-      <c r="C3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" t="n">
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
         <v>-0.1191417440227731</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>-0.2455113417974512</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3">
         <v>-0.09691680717176694</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3">
         <v>-0.2244983794870531</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3">
         <v>-0.07773792390383803</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3">
         <v>-0.1414474473507824</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J3">
         <v>-0.296709297971328</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3">
         <v>0.1188368149337552</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L3">
         <v>-0.08568571153207107</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M3">
         <v>0.007535366125411684</v>
       </c>
-      <c r="N3" t="n">
+      <c r="N3">
         <v>-0.007160999403591629</v>
       </c>
-      <c r="O3" t="n">
+      <c r="O3">
         <v>0.1490236447405327</v>
       </c>
-      <c r="P3" t="n">
+      <c r="P3">
         <v>0.1662874038639158</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="Q3">
         <v>-0.08594986830686391</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>3C04</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+    <row r="4" spans="1:17">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4">
         <v>-0.1121271029347614</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4">
         <v>-0.1191417440227731</v>
       </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="n">
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
         <v>-0.06009322247878907</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4">
         <v>-0.04882833750087008</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4">
         <v>-0.1148070794193453</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4">
         <v>-0.1422465090391772</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4">
         <v>0.1368754114967538</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J4">
         <v>-0.006559615325480292</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4">
         <v>-0.2070892027018655</v>
       </c>
-      <c r="L4" t="n">
+      <c r="L4">
         <v>-0.1673484710603782</v>
       </c>
-      <c r="M4" t="n">
+      <c r="M4">
         <v>-0.1908375596530751</v>
       </c>
-      <c r="N4" t="n">
+      <c r="N4">
         <v>0.02277801587682716</v>
       </c>
-      <c r="O4" t="n">
+      <c r="O4">
         <v>0.1138291393811654</v>
       </c>
-      <c r="P4" t="n">
+      <c r="P4">
         <v>0.06191290237945385</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="Q4">
         <v>0.1884136482881426</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>3C05</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+    <row r="5" spans="1:17">
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5">
         <v>0.01467795809162198</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5">
         <v>-0.2455113417974512</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5">
         <v>-0.06009322247878907</v>
       </c>
-      <c r="E5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" t="n">
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
         <v>-0.1178072027104749</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5">
         <v>-0.1876994294801837</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5">
         <v>0.02182926675817642</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5">
         <v>-0.003052786262868995</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J5">
         <v>-0.1499232532119751</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5">
         <v>-0.0221449161701662</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L5">
         <v>-0.02148986210338777</v>
       </c>
-      <c r="M5" t="n">
+      <c r="M5">
         <v>-0.1292912195276677</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N5">
         <v>-0.3094839627488249</v>
       </c>
-      <c r="O5" t="n">
+      <c r="O5">
         <v>-0.09122359089304791</v>
       </c>
-      <c r="P5" t="n">
+      <c r="P5">
         <v>0.002836296738229003</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="Q5">
         <v>-0.07852745019519748</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>3C06</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+    <row r="6" spans="1:17">
+      <c r="A6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6">
         <v>-0.0998038780137567</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6">
         <v>-0.09691680717176694</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6">
         <v>-0.04882833750087008</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6">
         <v>-0.1178072027104749</v>
       </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" t="n">
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
         <v>0.07382492338942878</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6">
         <v>-0.1159768973323803</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I6">
         <v>-0.03771319583001898</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J6">
         <v>-0.05226600544908928</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K6">
         <v>-0.2291802028326535</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L6">
         <v>-0.07318861530284203</v>
       </c>
-      <c r="M6" t="n">
+      <c r="M6">
         <v>-0.09911061060217946</v>
       </c>
-      <c r="N6" t="n">
+      <c r="N6">
         <v>-0.01146657058055237</v>
       </c>
-      <c r="O6" t="n">
+      <c r="O6">
         <v>0.08381548315694157</v>
       </c>
-      <c r="P6" t="n">
+      <c r="P6">
         <v>-0.1507574273350401</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="Q6">
         <v>-0.1736927683548675</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>3C07</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+    <row r="7" spans="1:17">
+      <c r="A7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7">
         <v>-0.2055615731357613</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7">
         <v>-0.2244983794870531</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7">
         <v>-0.1148070794193453</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7">
         <v>-0.1876994294801837</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7">
         <v>0.07382492338942878</v>
       </c>
-      <c r="G7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" t="n">
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
         <v>0.2886006104806107</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7">
         <v>0.2425958643480183</v>
       </c>
-      <c r="J7" t="n">
+      <c r="J7">
         <v>0.04027099777961001</v>
       </c>
-      <c r="K7" t="n">
+      <c r="K7">
         <v>0.05108810170416033</v>
       </c>
-      <c r="L7" t="n">
+      <c r="L7">
         <v>-0.08875702602600159</v>
       </c>
-      <c r="M7" t="n">
+      <c r="M7">
         <v>0.04119811351603456</v>
       </c>
-      <c r="N7" t="n">
+      <c r="N7">
         <v>0.07264767665402652</v>
       </c>
-      <c r="O7" t="n">
+      <c r="O7">
         <v>-0.2698683067481655</v>
       </c>
-      <c r="P7" t="n">
+      <c r="P7">
         <v>-0.2540710351998539</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="Q7">
         <v>0.01075244966787154</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>3C08</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+    <row r="8" spans="1:17">
+      <c r="A8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8">
         <v>0.03873230532879787</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8">
         <v>-0.07773792390383803</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8">
         <v>-0.1422465090391772</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8">
         <v>0.02182926675817642</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8">
         <v>-0.1159768973323803</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8">
         <v>0.2886006104806107</v>
       </c>
-      <c r="H8" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" t="n">
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
         <v>0.02650128489944373</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J8">
         <v>-0.01176377492315518</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K8">
         <v>0.1273190193871465</v>
       </c>
-      <c r="L8" t="n">
+      <c r="L8">
         <v>-0.06224377527247782</v>
       </c>
-      <c r="M8" t="n">
+      <c r="M8">
         <v>0.02811851070690768</v>
       </c>
-      <c r="N8" t="n">
+      <c r="N8">
         <v>-0.09393007103567844</v>
       </c>
-      <c r="O8" t="n">
+      <c r="O8">
         <v>-0.145736920675665</v>
       </c>
-      <c r="P8" t="n">
+      <c r="P8">
         <v>-0.2909816191067932</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="Q8">
         <v>-0.1747526967162389</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>3C09</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+    <row r="9" spans="1:17">
+      <c r="A9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9">
         <v>0.002201016425689495</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9">
         <v>-0.1414474473507824</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9">
         <v>0.1368754114967538</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9">
         <v>-0.003052786262868995</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9">
         <v>-0.03771319583001898</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9">
         <v>0.2425958643480183</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H9">
         <v>0.02650128489944373</v>
       </c>
-      <c r="I9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" t="n">
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
         <v>-0.0002709456394808113</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K9">
         <v>0.06589816625386424</v>
       </c>
-      <c r="L9" t="n">
+      <c r="L9">
         <v>-0.2904590872753287</v>
       </c>
-      <c r="M9" t="n">
+      <c r="M9">
         <v>-0.01832707448533353</v>
       </c>
-      <c r="N9" t="n">
+      <c r="N9">
         <v>-0.2089028351790923</v>
       </c>
-      <c r="O9" t="n">
+      <c r="O9">
         <v>-0.07171277848532429</v>
       </c>
-      <c r="P9" t="n">
+      <c r="P9">
         <v>-0.2691371102555323</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="Q9">
         <v>0.07782862552723248</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>3C10</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+    <row r="10" spans="1:17">
+      <c r="A10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10">
         <v>-0.1213430151999095</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10">
         <v>-0.296709297971328</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10">
         <v>-0.006559615325480292</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10">
         <v>-0.1499232532119751</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10">
         <v>-0.05226600544908928</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10">
         <v>0.04027099777961001</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H10">
         <v>-0.01176377492315518</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I10">
         <v>-0.0002709456394808113</v>
       </c>
-      <c r="J10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" t="n">
+      <c r="J10">
+        <v>1</v>
+      </c>
+      <c r="K10">
         <v>-0.1461322510155612</v>
       </c>
-      <c r="L10" t="n">
+      <c r="L10">
         <v>-0.05944285842542523</v>
       </c>
-      <c r="M10" t="n">
+      <c r="M10">
         <v>-0.1862617857690863</v>
       </c>
-      <c r="N10" t="n">
+      <c r="N10">
         <v>0.07279000173627602</v>
       </c>
-      <c r="O10" t="n">
+      <c r="O10">
         <v>-0.06043381521329393</v>
       </c>
-      <c r="P10" t="n">
+      <c r="P10">
         <v>-0.2240372015906962</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="Q10">
         <v>0.08355394807753153</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>3C11</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
+    <row r="11" spans="1:17">
+      <c r="A11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11">
         <v>0.06225760883671789</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11">
         <v>0.1188368149337552</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11">
         <v>-0.2070892027018655</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11">
         <v>-0.0221449161701662</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11">
         <v>-0.2291802028326535</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11">
         <v>0.05108810170416033</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H11">
         <v>0.1273190193871465</v>
       </c>
-      <c r="I11" t="n">
+      <c r="I11">
         <v>0.06589816625386424</v>
       </c>
-      <c r="J11" t="n">
+      <c r="J11">
         <v>-0.1461322510155612</v>
       </c>
-      <c r="K11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L11" t="n">
+      <c r="K11">
+        <v>1</v>
+      </c>
+      <c r="L11">
         <v>0.1154047276970864</v>
       </c>
-      <c r="M11" t="n">
+      <c r="M11">
         <v>0.03322793400622095</v>
       </c>
-      <c r="N11" t="n">
+      <c r="N11">
         <v>-0.09018226581114357</v>
       </c>
-      <c r="O11" t="n">
+      <c r="O11">
         <v>-0.1937296307683508</v>
       </c>
-      <c r="P11" t="n">
+      <c r="P11">
         <v>-0.215183275041049</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="Q11">
         <v>0.01407095909662935</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>3C12</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
+    <row r="12" spans="1:17">
+      <c r="A12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12">
         <v>-0.231502533472337</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12">
         <v>-0.08568571153207107</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12">
         <v>-0.1673484710603782</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12">
         <v>-0.02148986210338777</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12">
         <v>-0.07318861530284203</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12">
         <v>-0.08875702602600159</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H12">
         <v>-0.06224377527247782</v>
       </c>
-      <c r="I12" t="n">
+      <c r="I12">
         <v>-0.2904590872753287</v>
       </c>
-      <c r="J12" t="n">
+      <c r="J12">
         <v>-0.05944285842542523</v>
       </c>
-      <c r="K12" t="n">
+      <c r="K12">
         <v>0.1154047276970864</v>
       </c>
-      <c r="L12" t="n">
-        <v>1</v>
-      </c>
-      <c r="M12" t="n">
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12">
         <v>-0.01525588458923418</v>
       </c>
-      <c r="N12" t="n">
+      <c r="N12">
         <v>-0.1294020065613939</v>
       </c>
-      <c r="O12" t="n">
+      <c r="O12">
         <v>-0.1986369316515291</v>
       </c>
-      <c r="P12" t="n">
+      <c r="P12">
         <v>0.02679930162498</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="Q12">
         <v>-0.1278492510854517</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>3C13</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
+    <row r="13" spans="1:17">
+      <c r="A13" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13">
         <v>0.0622219564254666</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13">
         <v>0.007535366125411684</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13">
         <v>-0.1908375596530751</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13">
         <v>-0.1292912195276677</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13">
         <v>-0.09911061060217946</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13">
         <v>0.04119811351603456</v>
       </c>
-      <c r="H13" t="n">
+      <c r="H13">
         <v>0.02811851070690768</v>
       </c>
-      <c r="I13" t="n">
+      <c r="I13">
         <v>-0.01832707448533353</v>
       </c>
-      <c r="J13" t="n">
+      <c r="J13">
         <v>-0.1862617857690863</v>
       </c>
-      <c r="K13" t="n">
+      <c r="K13">
         <v>0.03322793400622095</v>
       </c>
-      <c r="L13" t="n">
+      <c r="L13">
         <v>-0.01525588458923418</v>
       </c>
-      <c r="M13" t="n">
-        <v>1</v>
-      </c>
-      <c r="N13" t="n">
+      <c r="M13">
+        <v>1</v>
+      </c>
+      <c r="N13">
         <v>-0.2062005029734034</v>
       </c>
-      <c r="O13" t="n">
+      <c r="O13">
         <v>-0.1030688683106085</v>
       </c>
-      <c r="P13" t="n">
+      <c r="P13">
         <v>-0.1269891042405047</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="Q13">
         <v>-0.09420578225387052</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>3C14</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
+    <row r="14" spans="1:17">
+      <c r="A14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14">
         <v>-0.07143255158646721</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14">
         <v>-0.007160999403591629</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14">
         <v>0.02277801587682716</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14">
         <v>-0.3094839627488249</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14">
         <v>-0.01146657058055237</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14">
         <v>0.07264767665402652</v>
       </c>
-      <c r="H14" t="n">
+      <c r="H14">
         <v>-0.09393007103567844</v>
       </c>
-      <c r="I14" t="n">
+      <c r="I14">
         <v>-0.2089028351790923</v>
       </c>
-      <c r="J14" t="n">
+      <c r="J14">
         <v>0.07279000173627602</v>
       </c>
-      <c r="K14" t="n">
+      <c r="K14">
         <v>-0.09018226581114357</v>
       </c>
-      <c r="L14" t="n">
+      <c r="L14">
         <v>-0.1294020065613939</v>
       </c>
-      <c r="M14" t="n">
+      <c r="M14">
         <v>-0.2062005029734034</v>
       </c>
-      <c r="N14" t="n">
-        <v>1</v>
-      </c>
-      <c r="O14" t="n">
+      <c r="N14">
+        <v>1</v>
+      </c>
+      <c r="O14">
         <v>-0.02648425848632626</v>
       </c>
-      <c r="P14" t="n">
+      <c r="P14">
         <v>-0.02290830842563061</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="Q14">
         <v>-0.0982251113470939</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>3C15</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
+    <row r="15" spans="1:17">
+      <c r="A15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15">
         <v>0.2287020214566456</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15">
         <v>0.1490236447405327</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15">
         <v>0.1138291393811654</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15">
         <v>-0.09122359089304791</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15">
         <v>0.08381548315694157</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15">
         <v>-0.2698683067481655</v>
       </c>
-      <c r="H15" t="n">
+      <c r="H15">
         <v>-0.145736920675665</v>
       </c>
-      <c r="I15" t="n">
+      <c r="I15">
         <v>-0.07171277848532429</v>
       </c>
-      <c r="J15" t="n">
+      <c r="J15">
         <v>-0.06043381521329393</v>
       </c>
-      <c r="K15" t="n">
+      <c r="K15">
         <v>-0.1937296307683508</v>
       </c>
-      <c r="L15" t="n">
+      <c r="L15">
         <v>-0.1986369316515291</v>
       </c>
-      <c r="M15" t="n">
+      <c r="M15">
         <v>-0.1030688683106085</v>
       </c>
-      <c r="N15" t="n">
+      <c r="N15">
         <v>-0.02648425848632626</v>
       </c>
-      <c r="O15" t="n">
-        <v>1</v>
-      </c>
-      <c r="P15" t="n">
+      <c r="O15">
+        <v>1</v>
+      </c>
+      <c r="P15">
         <v>0.04078723970581077</v>
       </c>
-      <c r="Q15" t="n">
+      <c r="Q15">
         <v>-0.3357235214201097</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>3C16</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
+    <row r="16" spans="1:17">
+      <c r="A16" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16">
         <v>-0.0286133563571018</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16">
         <v>0.1662874038639158</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16">
         <v>0.06191290237945385</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16">
         <v>0.002836296738229003</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16">
         <v>-0.1507574273350401</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16">
         <v>-0.2540710351998539</v>
       </c>
-      <c r="H16" t="n">
+      <c r="H16">
         <v>-0.2909816191067932</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I16">
         <v>-0.2691371102555323</v>
       </c>
-      <c r="J16" t="n">
+      <c r="J16">
         <v>-0.2240372015906962</v>
       </c>
-      <c r="K16" t="n">
+      <c r="K16">
         <v>-0.215183275041049</v>
       </c>
-      <c r="L16" t="n">
+      <c r="L16">
         <v>0.02679930162498</v>
       </c>
-      <c r="M16" t="n">
+      <c r="M16">
         <v>-0.1269891042405047</v>
       </c>
-      <c r="N16" t="n">
+      <c r="N16">
         <v>-0.02290830842563061</v>
       </c>
-      <c r="O16" t="n">
+      <c r="O16">
         <v>0.04078723970581077</v>
       </c>
-      <c r="P16" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q16" t="n">
+      <c r="P16">
+        <v>1</v>
+      </c>
+      <c r="Q16">
         <v>-0.1059528067654508</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>3C17</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
+    <row r="17" spans="1:17">
+      <c r="A17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17">
         <v>-0.1376742995782222</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17">
         <v>-0.08594986830686391</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17">
         <v>0.1884136482881426</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17">
         <v>-0.07852745019519748</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17">
         <v>-0.1736927683548675</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17">
         <v>0.01075244966787154</v>
       </c>
-      <c r="H17" t="n">
+      <c r="H17">
         <v>-0.1747526967162389</v>
       </c>
-      <c r="I17" t="n">
+      <c r="I17">
         <v>0.07782862552723248</v>
       </c>
-      <c r="J17" t="n">
+      <c r="J17">
         <v>0.08355394807753153</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K17">
         <v>0.01407095909662935</v>
       </c>
-      <c r="L17" t="n">
+      <c r="L17">
         <v>-0.1278492510854517</v>
       </c>
-      <c r="M17" t="n">
+      <c r="M17">
         <v>-0.09420578225387052</v>
       </c>
-      <c r="N17" t="n">
+      <c r="N17">
         <v>-0.0982251113470939</v>
       </c>
-      <c r="O17" t="n">
+      <c r="O17">
         <v>-0.3357235214201097</v>
       </c>
-      <c r="P17" t="n">
+      <c r="P17">
         <v>-0.1059528067654508</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="Q17">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>